<commit_message>
Remover sabor morango do pedido manual
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pCebD3AqGMmAWDpwcHAsR
</commit_message>
<xml_diff>
--- a/entregas/Solcitação Retirada - Pedido Manual.xlsx
+++ b/entregas/Solcitação Retirada - Pedido Manual.xlsx
@@ -656,7 +656,7 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>PRD-QTZ-RTD-00750-201</t>
+          <t>PRD-QTZ-RTD-00750-301</t>
         </is>
       </c>
       <c r="B7" s="20" t="n">
@@ -666,14 +666,8 @@
       <c r="D7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>PRD-QTZ-RTD-00750-301</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>6</v>
-      </c>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="4" t="n"/>
     </row>

</xml_diff>